<commit_message>
updated the 52 codes sheet
</commit_message>
<xml_diff>
--- a/results/review/52_codes_review.xlsx
+++ b/results/review/52_codes_review.xlsx
@@ -793,7 +793,7 @@
     <t xml:space="preserve">Mappings produced</t>
   </si>
   <si>
-    <t xml:space="preserve">Mappings for the 52 codes</t>
+    <t xml:space="preserve">False positives from the 52 codes</t>
   </si>
   <si>
     <t xml:space="preserve">Correct pairs to find</t>
@@ -14824,7 +14824,7 @@
   </sheetData>
   <autoFilter ref="A1:P241"/>
   <conditionalFormatting sqref="J2:J241">
-    <cfRule type="colorScale" priority="8">
+    <cfRule type="colorScale" priority="7">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -14836,7 +14836,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M2:M241">
-    <cfRule type="colorScale" priority="7">
+    <cfRule type="colorScale" priority="6">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -14848,7 +14848,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N2:N241">
-    <cfRule type="colorScale" priority="6">
+    <cfRule type="colorScale" priority="5">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -14860,7 +14860,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O2:O241">
-    <cfRule type="colorScale" priority="5">
+    <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -14872,7 +14872,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P2:P241">
-    <cfRule type="colorScale" priority="4">
+    <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -14884,7 +14884,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K2:K241">
-    <cfRule type="colorScale" priority="3">
+    <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -14896,18 +14896,6 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L2:L241">
-    <cfRule type="colorScale" priority="2">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H2:H241">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>

</xml_diff>